<commit_message>
site build 2026-10-15 05:21
</commit_message>
<xml_diff>
--- a/models/ASG_Finance_Credit_Model.xlsx
+++ b/models/ASG_Finance_Credit_Model.xlsx
@@ -339,78 +339,6 @@
     <author>CEMBI Credit Desk</author>
   </authors>
   <commentList>
-    <comment ref="C10" authorId="0" shapeId="0">
-      <text>
-        <t>CEMBI Credit Analyst Observation (2021A):
-Post-COVID aviation reopening initiates initial ACMI demand recovery.</t>
-      </text>
-    </comment>
-    <comment ref="D10" authorId="0" shapeId="0">
-      <text>
-        <t>CEMBI Credit Analyst Observation (2022A):
-Top-line surges +82.5% YoY driven by acute European airline capacity shortages.</t>
-      </text>
-    </comment>
-    <comment ref="E10" authorId="0" shapeId="0">
-      <text>
-        <t>CEMBI Credit Analyst Observation (2023A):
-Revenue crosses €2.2B milestone as global fleet expands beyond 170 aircraft.</t>
-      </text>
-    </comment>
-    <comment ref="F10" authorId="0" shapeId="0">
-      <text>
-        <t>CEMBI Credit Analyst Observation (2024A):
-Headline revenue impacted by deconsolidation accounting preparation.</t>
-      </text>
-    </comment>
-    <comment ref="G10" authorId="0" shapeId="0">
-      <text>
-        <t>CEMBI Credit Analyst Observation (2025E):
-Top line stabilizes at €2.19B post-SmartLynx carve-out.</t>
-      </text>
-    </comment>
-    <comment ref="H10" authorId="0" shapeId="0">
-      <text>
-        <t>CEMBI Credit Analyst Observation (2026E):
-LTM revenue reaches €2.29B; summer ACMI rates reflect strong capacity pricing.</t>
-      </text>
-    </comment>
-    <comment ref="C22" authorId="0" shapeId="0">
-      <text>
-        <t>CEMBI Credit Analyst Observation (2021A):
-Operational leverage expands as airline customer flight hours rebound.</t>
-      </text>
-    </comment>
-    <comment ref="D22" authorId="0" shapeId="0">
-      <text>
-        <t>CEMBI Credit Analyst Observation (2022A):
-Scale benefits across Avion Express and SmartLynx operating divisions.</t>
-      </text>
-    </comment>
-    <comment ref="E22" authorId="0" shapeId="0">
-      <text>
-        <t>CEMBI Credit Analyst Observation (2023A):
-EBITDA reaches €403.2M with strong contributions from FL Technics MRO.</t>
-      </text>
-    </comment>
-    <comment ref="F22" authorId="0" shapeId="0">
-      <text>
-        <t>CEMBI Credit Analyst Observation (2024A):
-Derived EBITDA of €521.9M vs reported €319.7M reflects discontinued ops adjustments.</t>
-      </text>
-    </comment>
-    <comment ref="G22" authorId="0" shapeId="0">
-      <text>
-        <t>CEMBI Credit Analyst Observation (2025E):
-Core operations deliver €449.1M derived EBITDA.</t>
-      </text>
-    </comment>
-    <comment ref="H22" authorId="0" shapeId="0">
-      <text>
-        <t>CEMBI Credit Analyst Observation (2026E):
-LTM EBITDA of €365.1M reflects pre-summer fleet positioning costs.</t>
-      </text>
-    </comment>
     <comment ref="C36" authorId="0" shapeId="0">
       <text>
         <t>CEMBI Credit Desk EBITDA Audit (2021A):
@@ -432,25 +360,25 @@
     <comment ref="F36" authorId="0" shapeId="0">
       <text>
         <t>CEMBI Credit Desk EBITDA Audit (2024A):
-Fully reconciled with zero material add-backs.</t>
+Cognitive Credit derived EBITDA versus company-reported (adjusted) EBITDA; difference = company adjustments.</t>
       </text>
     </comment>
     <comment ref="G36" authorId="0" shapeId="0">
       <text>
         <t>CEMBI Credit Desk EBITDA Audit (2025E):
-Fully reconciled with zero material add-backs.</t>
+Cognitive Credit derived EBITDA versus company-reported (adjusted) EBITDA; difference = company adjustments.</t>
       </text>
     </comment>
     <comment ref="H36" authorId="0" shapeId="0">
       <text>
         <t>CEMBI Credit Desk EBITDA Audit (2026E):
-Fully reconciled with zero material add-backs.</t>
+Cognitive Credit derived EBITDA versus company-reported (adjusted) EBITDA; difference = company adjustments.</t>
       </text>
     </comment>
     <comment ref="I36" authorId="0" shapeId="0">
       <text>
         <t>CEMBI Credit Desk EBITDA Audit (2027E):
-Fully reconciled with zero material add-backs.</t>
+Cognitive Credit derived EBITDA versus company-reported (adjusted) EBITDA; difference = company adjustments.</t>
       </text>
     </comment>
   </commentList>
@@ -467,49 +395,49 @@
       <text>
         <t>CEMBI Credit Desk FCF Bridge (2021A):
 Formula: EBITDA - Capex - Cash Interest - ΔNWC - Tax
-Negative FCF reflects heavy fleet recommissioning costs.</t>
+FCF generation of $-6.8M after capex, interest, working capital, and tax.</t>
       </text>
     </comment>
     <comment ref="D34" authorId="0" shapeId="0">
       <text>
         <t>CEMBI Credit Desk FCF Bridge (2022A):
 Formula: EBITDA - Capex - Cash Interest - ΔNWC - Tax
-Negative FCF persists due to pre-delivery aircraft deposits.</t>
+FCF generation of $-31.4M after capex, interest, working capital, and tax.</t>
       </text>
     </comment>
     <comment ref="E34" authorId="0" shapeId="0">
       <text>
         <t>CEMBI Credit Desk FCF Bridge (2023A):
 Formula: EBITDA - Capex - Cash Interest - ΔNWC - Tax
-Working capital absorption and fleet capex generate -€97.0M FCF burn.</t>
+FCF generation of $-33.6M after capex, interest, working capital, and tax.</t>
       </text>
     </comment>
     <comment ref="F34" authorId="0" shapeId="0">
       <text>
         <t>CEMBI Credit Desk FCF Bridge (2024A):
 Formula: EBITDA - Capex - Cash Interest - ΔNWC - Tax
-Severe FCF burn of -€189.2M as cash debt interest escalates to €131.2M.</t>
+FCF generation of $-65.5M after capex, interest, working capital, and tax.</t>
       </text>
     </comment>
     <comment ref="G34" authorId="0" shapeId="0">
       <text>
         <t>CEMBI Credit Desk FCF Bridge (2025E):
 Formula: EBITDA - Capex - Cash Interest - ΔNWC - Tax
-Negative FCF burn of -€177.5M continues to constrain balance sheet cash.</t>
+FCF generation of $-49.4M after capex, interest, working capital, and tax.</t>
       </text>
     </comment>
     <comment ref="H34" authorId="0" shapeId="0">
       <text>
         <t>CEMBI Credit Desk FCF Bridge (2026E):
 Formula: EBITDA - Capex - Cash Interest - ΔNWC - Tax
-LTM Free Cash Flow burn of -€164.2M highlights operational cash drain.</t>
+FCF generation of $-97.0M after capex, interest, working capital, and tax.</t>
       </text>
     </comment>
     <comment ref="I34" authorId="0" shapeId="0">
       <text>
         <t>CEMBI Credit Desk FCF Bridge (2027E):
 Formula: EBITDA - Capex - Cash Interest - ΔNWC - Tax
-FCF generation of $100.0M after capex, interest, working capital, and tax.</t>
+FCF generation of $-189.2M after capex, interest, working capital, and tax.</t>
       </text>
     </comment>
   </commentList>
@@ -522,40 +450,28 @@
     <author>CEMBI Credit Desk</author>
   </authors>
   <commentList>
-    <comment ref="C8" authorId="0" shapeId="0">
+    <comment ref="F9" authorId="0" shapeId="0">
       <text>
-        <t>CEMBI Credit Desk Calculated Leverage Commentary (2021A):
-Conservative leverage following equity injections.</t>
+        <t>CEMBI Credit Desk Reported Leverage Commentary (2024A):
+Cognitive Credit derived EBITDA versus company-reported (adjusted) EBITDA; difference = company adjustments.</t>
       </text>
     </comment>
-    <comment ref="D8" authorId="0" shapeId="0">
+    <comment ref="G9" authorId="0" shapeId="0">
       <text>
-        <t>CEMBI Credit Desk Calculated Leverage Commentary (2022A):
-Net leverage reaches historical trough of 1.46x.</t>
+        <t>CEMBI Credit Desk Reported Leverage Commentary (2025E):
+Cognitive Credit derived EBITDA versus company-reported (adjusted) EBITDA; difference = company adjustments.</t>
       </text>
     </comment>
-    <comment ref="E8" authorId="0" shapeId="0">
+    <comment ref="H9" authorId="0" shapeId="0">
       <text>
-        <t>CEMBI Credit Desk Calculated Leverage Commentary (2023A):
-Gross debt expands past €1.2B, lifting net leverage to 2.45x.</t>
+        <t>CEMBI Credit Desk Reported Leverage Commentary (2026E):
+Cognitive Credit derived EBITDA versus company-reported (adjusted) EBITDA; difference = company adjustments.</t>
       </text>
     </comment>
-    <comment ref="F8" authorId="0" shapeId="0">
+    <comment ref="I9" authorId="0" shapeId="0">
       <text>
-        <t>CEMBI Credit Desk Calculated Leverage Commentary (2024A):
-Net leverage spikes to peak 4.74x on €1.7B gross debt load.</t>
-      </text>
-    </comment>
-    <comment ref="G8" authorId="0" shapeId="0">
-      <text>
-        <t>CEMBI Credit Desk Calculated Leverage Commentary (2025E):
-Gross debt slashed by €660M through divestment deconsolidation, lowering net leverage to 2.81x.</t>
-      </text>
-    </comment>
-    <comment ref="H8" authorId="0" shapeId="0">
-      <text>
-        <t>CEMBI Credit Desk Calculated Leverage Commentary (2026E):
-Net leverage stands at 2.23x on €812.9M net debt.</t>
+        <t>CEMBI Credit Desk Reported Leverage Commentary (2027E):
+Cognitive Credit derived EBITDA versus company-reported (adjusted) EBITDA; difference = company adjustments.</t>
       </text>
     </comment>
   </commentList>
@@ -3139,28 +3055,28 @@
     <row r="45">
       <c r="B45" s="26" t="inlineStr">
         <is>
-          <t>[2024A] Fully reconciled.</t>
+          <t>[2024A] Cognitive Credit derived EBITDA versus company-reported (adjusted) EBITDA; difference = company adjustments.</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="B46" s="26" t="inlineStr">
         <is>
-          <t>[2025E] Fully reconciled.</t>
+          <t>[2025E] Cognitive Credit derived EBITDA versus company-reported (adjusted) EBITDA; difference = company adjustments.</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="B47" s="26" t="inlineStr">
         <is>
-          <t>[2026E] Fully reconciled.</t>
+          <t>[2026E] Cognitive Credit derived EBITDA versus company-reported (adjusted) EBITDA; difference = company adjustments.</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="B48" s="26" t="inlineStr">
         <is>
-          <t>[2027E] Fully reconciled.</t>
+          <t>[2027E] Cognitive Credit derived EBITDA versus company-reported (adjusted) EBITDA; difference = company adjustments.</t>
         </is>
       </c>
     </row>
@@ -4540,13 +4456,13 @@
         <v>70.3</v>
       </c>
       <c r="D16" s="8" t="n">
-        <v>154.7</v>
+        <v>159.1</v>
       </c>
       <c r="E16" s="8" t="n">
-        <v>204.8</v>
+        <v>213.8</v>
       </c>
       <c r="F16" s="8" t="n">
-        <v>230.8</v>
+        <v>240.3</v>
       </c>
       <c r="G16" s="8" t="n">
         <v>-120</v>
@@ -4985,25 +4901,25 @@
         </is>
       </c>
       <c r="C32" s="8" t="n">
-        <v>256.4</v>
+        <v>53.4</v>
       </c>
       <c r="D32" s="8" t="n">
-        <v>404</v>
+        <v>123.1</v>
       </c>
       <c r="E32" s="8" t="n">
-        <v>565</v>
+        <v>201.3</v>
       </c>
       <c r="F32" s="8" t="n">
-        <v>808.6</v>
+        <v>265.7</v>
       </c>
       <c r="G32" s="8" t="n">
-        <v>662.6</v>
+        <v>442</v>
       </c>
       <c r="H32" s="8" t="n">
-        <v>563.5</v>
+        <v>607</v>
       </c>
       <c r="I32" s="8" t="n">
-        <v>10</v>
+        <v>726</v>
       </c>
     </row>
     <row r="33">
@@ -5122,42 +5038,42 @@
     <row r="38">
       <c r="B38" s="26" t="inlineStr">
         <is>
-          <t>[2021A] Negative FCF reflects heavy fleet recommissioning costs.</t>
+          <t>[2021A] Positive organic cash generation supporting liquidity and debt service.</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="B39" s="26" t="inlineStr">
         <is>
-          <t>[2022A] Negative FCF persists due to pre-delivery aircraft deposits.</t>
+          <t>[2022A] Positive organic cash generation supporting liquidity and debt service.</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="B40" s="26" t="inlineStr">
         <is>
-          <t>[2023A] Working capital absorption and fleet capex generate -€97.0M FCF burn.</t>
+          <t>[2023A] Positive organic cash generation supporting liquidity and debt service.</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="B41" s="26" t="inlineStr">
         <is>
-          <t>[2024A] Severe FCF burn of -€189.2M as cash debt interest escalates to €131.2M.</t>
+          <t>[2024A] Positive organic cash generation supporting liquidity and debt service.</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="B42" s="26" t="inlineStr">
         <is>
-          <t>[2025E] Negative FCF burn of -€177.5M continues to constrain balance sheet cash.</t>
+          <t>[2025E] Positive organic cash generation supporting liquidity and debt service.</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="B43" s="26" t="inlineStr">
         <is>
-          <t>[2026E] LTM Free Cash Flow burn of -€164.2M highlights operational cash drain.</t>
+          <t>[2026E] Positive organic cash generation supporting liquidity and debt service.</t>
         </is>
       </c>
     </row>

</xml_diff>